<commit_message>
Update Excel task entries
</commit_message>
<xml_diff>
--- a/docs/sweng/Projektplan.xlsx
+++ b/docs/sweng/Projektplan.xlsx
@@ -5,10 +5,10 @@
   <workbookPr dateCompatibility="0" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6bca3ab9c796c159/Dokumente/ZUniversity/HS26/SoftwareEngineering/Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\IdeaProjects\ForgeSynesisHS26\docs\sweng\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8_{FC8D6FDA-7439-4BF3-8F86-92206165D753}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{D22E4981-959E-4BDE-B3D6-AC340D6F4F96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{01424205-40D3-491C-9A3E-5D7E838D4391}"/>
   </bookViews>
@@ -42,14 +42,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="38" uniqueCount="35">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="49" uniqueCount="49">
   <si>
     <t>ID</t>
   </si>
   <si>
-    <t>Phase/ Tasks</t>
-  </si>
-  <si>
     <t>Entwickler</t>
   </si>
   <si>
@@ -83,9 +80,6 @@
     <t>T09</t>
   </si>
   <si>
-    <t>T10</t>
-  </si>
-  <si>
     <t>T11</t>
   </si>
   <si>
@@ -107,53 +101,101 @@
     <t>T17</t>
   </si>
   <si>
-    <t>T18</t>
-  </si>
-  <si>
-    <t>T19</t>
-  </si>
-  <si>
     <t>T20</t>
   </si>
   <si>
     <t>T21</t>
   </si>
   <si>
-    <t>T22</t>
-  </si>
-  <si>
-    <t>Anforderungengen und Projektumfang festlegen</t>
-  </si>
-  <si>
-    <t>Funktionale Anforderungen einzelner Tasks aufteilen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JabRef-Code und Erweiterungsmöglichkeiten untersuchen </t>
-  </si>
-  <si>
-    <t>Gemini API und andere Modelle untersuchen</t>
-  </si>
-  <si>
     <t>Erledigt</t>
   </si>
   <si>
     <t>Startdatum</t>
   </si>
   <si>
-    <t>Gemini API integrieren</t>
-  </si>
-  <si>
-    <t>Kategorie</t>
-  </si>
-  <si>
-    <t>Analyse</t>
+    <t xml:space="preserve">Fehlermeldung an Forge Synesis weiterleiten und korrekt abbilden </t>
+  </si>
+  <si>
+    <t>Funktionale und nicht-funktionale Anforderugen festlegen</t>
+  </si>
+  <si>
+    <t>Anforderungen und Abnahmekriterien im Pflichtenheft festlegen</t>
+  </si>
+  <si>
+    <t>JabRef-Code, Erweiterungspunkte und Buildprozesse untersuchen</t>
+  </si>
+  <si>
+    <t>Gemini API, Modelle und Machbarkeit untersuchen</t>
+  </si>
+  <si>
+    <t>Entwicklungsumgebung und Projekt einrichten und starten</t>
+  </si>
+  <si>
+    <t>Phase</t>
+  </si>
+  <si>
+    <t>Tasks</t>
+  </si>
+  <si>
+    <t>Architektur und Modularaufteilung für Forge Synesis entwerfen</t>
+  </si>
+  <si>
+    <t>Schnittstellen und Datenfluss zwischen JabRef, Forge Synesis und Gemini definieren</t>
+  </si>
+  <si>
+    <t>Git-Workflow, Branches und Integrationsregeln festlegen</t>
+  </si>
+  <si>
+    <t>Grundstruktur für Forge Synesis festlegen und in JabRef implementieren</t>
+  </si>
+  <si>
+    <t>Grundlegende Benutzeroberfläche entwerfen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Previewfenster implementieren </t>
+  </si>
+  <si>
+    <t>Auswahl des Lernmaterials implementieren</t>
+  </si>
+  <si>
+    <t>Einstellung der Parameter implementieren</t>
+  </si>
+  <si>
+    <t>Ladezustandsanzeige implementieren</t>
+  </si>
+  <si>
+    <t>Flashcards von Gemini nach Forge Synesis importieren und anzeigen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Testumgebung und Testframework einrichten </t>
+  </si>
+  <si>
+    <t xml:space="preserve">T10 </t>
+  </si>
+  <si>
+    <t>Sichere Konfiguration des API Schlüssels implementieren</t>
+  </si>
+  <si>
+    <t>Verbindung zu Gemini implementieren und Testanfragen durchführen</t>
+  </si>
+  <si>
+    <t>Lernmaterial für die Übergabe an Gemini vorbereiten</t>
+  </si>
+  <si>
+    <t>Prompt für die Generierung der Flashcards entwickeln</t>
+  </si>
+  <si>
+    <t>API Antwort verwerten und in Flashcard-Format übertragen</t>
+  </si>
+  <si>
+    <t>Generierte Karten in UI Anzeigen</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -163,6 +205,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -188,8 +238,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="10"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -524,10 +581,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3E3C109-C609-4D69-8FDF-866EE7A4456E}">
-  <dimension ref="A3:G25"/>
+  <dimension ref="A3:G29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="54.7109375" customWidth="1"/>
+    <col min="3" max="3" width="58.7109375" customWidth="1"/>
     <col min="4" max="4" width="26.7109375" customWidth="1"/>
     <col min="5" max="5" width="21.42578125" customWidth="1"/>
     <col min="6" max="6" width="57.140625" customWidth="1"/>
@@ -535,167 +592,319 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" t="s">
-        <v>31</v>
-      </c>
-      <c r="F3" t="s">
-        <v>2</v>
-      </c>
-      <c r="G3" t="s">
-        <v>30</v>
+      <c r="G3" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>34</v>
+        <v>2</v>
+      </c>
+      <c r="B4" s="2">
+        <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>24</v>
+      </c>
+      <c r="D4" s="3">
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="3">
         <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>34</v>
+        <v>4</v>
+      </c>
+      <c r="B6" s="2">
+        <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>26</v>
+      </c>
+      <c r="D6" s="3">
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" t="s">
-        <v>34</v>
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>27</v>
+      </c>
+      <c r="D7" s="3">
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>7</v>
+      </c>
+      <c r="B8" s="2">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="3">
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
+      <c r="B9" s="2"/>
+      <c r="D9" s="3"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>8</v>
+      </c>
+      <c r="B10" s="2">
+        <v>2</v>
+      </c>
+      <c r="C10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="3">
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>9</v>
+      </c>
+      <c r="B11" s="2">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="3">
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>10</v>
+      </c>
+      <c r="B12" s="2">
+        <v>2</v>
+      </c>
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="3">
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>11</v>
+      </c>
+      <c r="B13" s="2">
+        <v>2</v>
+      </c>
+      <c r="C13" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" s="3">
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>42</v>
+      </c>
+      <c r="B14" s="2">
+        <v>2</v>
+      </c>
+      <c r="C14" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="3">
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>15</v>
-      </c>
+      <c r="B15" s="2"/>
+      <c r="D15" s="3"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" s="2">
+        <v>3</v>
+      </c>
+      <c r="C16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="2">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" s="2">
+        <v>3</v>
+      </c>
+      <c r="C18" t="s">
+        <v>37</v>
+      </c>
+      <c r="D18" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" s="2">
+        <v>3</v>
+      </c>
+      <c r="C19" t="s">
+        <v>38</v>
+      </c>
+      <c r="D19" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="B20" s="2">
+        <v>3</v>
+      </c>
+      <c r="C20" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="B21" s="2">
+        <v>3</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>18</v>
       </c>
-      <c r="C18" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="B22" s="2">
+        <v>3</v>
+      </c>
+      <c r="C22" t="s">
+        <v>23</v>
+      </c>
+      <c r="D22" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B23" s="2"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B24" s="2"/>
+      <c r="C24" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="B25" s="2"/>
+      <c r="C25" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>25</v>
+      <c r="B26" s="2"/>
+      <c r="C26" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C27" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C28" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C29" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>